<commit_message>
add PCB version 2 layers no stitching via
</commit_message>
<xml_diff>
--- a/Generate Files/BOM/243-436_PCB-Support-STM32F407.xlsx
+++ b/Generate Files/BOM/243-436_PCB-Support-STM32F407.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lecegeplimoilou-my.sharepoint.com/personal/kevin_cotton_cegeplimoilou_ca/Documents/_Cours-TGE/243-436-Dev-Prod4-Certifications/kit/243-436-PCB-Support-STM32F407/Generate Files/BOM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lecegeplimoilou-my.sharepoint.com/personal/kevin_cotton_cegeplimoilou_ca/Documents/_Cours-TGE/243-436-Dev-Prod4-Certifications/laboratoires/Labo1-Kit-Developpement-STM32/243-436-PCB-Support-STM32F407/Generate Files/BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5F8C2CF-F05C-4C22-B06F-88959762D001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{F5F8C2CF-F05C-4C22-B06F-88959762D001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D13B841-24F7-4ECC-B6FF-F7F992A83DBD}"/>
   <bookViews>
-    <workbookView xWindow="516" yWindow="660" windowWidth="20772" windowHeight="11580" xr2:uid="{FDB7F961-E6FF-49A7-9223-DD31578ADDCC}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="20112" windowHeight="12048" xr2:uid="{FDB7F961-E6FF-49A7-9223-DD31578ADDCC}"/>
   </bookViews>
   <sheets>
     <sheet name="243-436_PCB-Support-STM32F407" sheetId="1" r:id="rId1"/>
@@ -587,7 +587,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -649,7 +649,9 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{5597E743-E45E-48C9-BCDA-53213608DDC2}"/>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>

</xml_diff>

<commit_message>
add option LDO regulator on rev.B
</commit_message>
<xml_diff>
--- a/Generate Files/BOM/243-436_PCB-Support-STM32F407.xlsx
+++ b/Generate Files/BOM/243-436_PCB-Support-STM32F407.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lecegeplimoilou-my.sharepoint.com/personal/kevin_cotton_cegeplimoilou_ca/Documents/_Cours-TGE/243-436-Dev-Prod4-Certifications/laboratoires/Labo1-Kit-Developpement-STM32/243-436-PCB-Support-STM32F407/Generate Files/BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E556556E-FEDB-4E74-A729-C2F99570CC24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4785766C-DEEF-4405-A4CA-9CD24D3A443C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{898CD67B-8DE6-472D-ACF8-2736EC8F45DD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{70CBCBFD-1FBA-45C6-825C-CDE4DBF0641D}"/>
   </bookViews>
   <sheets>
     <sheet name="243-436_PCB-Support-STM32F407" sheetId="1" r:id="rId1"/>
@@ -1085,7 +1085,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED8784F8-9DF7-4BCD-8ABB-BCA9217864F8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1A17B6D-D7B4-415C-B61D-4F9E9DD390CA}">
   <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>